<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-06-23 21:27:14
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -802,7 +802,7 @@
         </is>
       </c>
       <c r="L6" s="4" t="n">
-        <v>151</v>
+        <v>153</v>
       </c>
     </row>
     <row r="7">
@@ -853,7 +853,7 @@
         </is>
       </c>
       <c r="L7" s="4" t="n">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
     <row r="8">
@@ -964,7 +964,7 @@
       </c>
       <c r="L9" s="4" t="inlineStr">
         <is>
-          <t>47.0%</t>
+          <t>47.7%</t>
         </is>
       </c>
     </row>
@@ -1021,7 +1021,7 @@
       </c>
       <c r="L10" s="4" t="inlineStr">
         <is>
-          <t>80.7%</t>
+          <t>80.4%</t>
         </is>
       </c>
     </row>
@@ -1806,22 +1806,22 @@
         <v>40</v>
       </c>
       <c r="O21" s="4" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="P21" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Q21" s="4" t="n">
         <v>16</v>
       </c>
       <c r="R21" s="4" t="inlineStr">
         <is>
-          <t>52.5%</t>
+          <t>55.0%</t>
         </is>
       </c>
       <c r="S21" s="4" t="inlineStr">
         <is>
-          <t>86.3%</t>
+          <t>86.6%</t>
         </is>
       </c>
     </row>
@@ -1884,22 +1884,22 @@
         <v>40</v>
       </c>
       <c r="O22" s="4" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="P22" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Q22" s="4" t="n">
         <v>16</v>
       </c>
       <c r="R22" s="4" t="inlineStr">
         <is>
-          <t>52.5%</t>
+          <t>55.0%</t>
         </is>
       </c>
       <c r="S22" s="4" t="inlineStr">
         <is>
-          <t>78.6%</t>
+          <t>75.8%</t>
         </is>
       </c>
     </row>
@@ -9677,7 +9677,7 @@
       </c>
       <c r="G195" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 160715@med.asu.edu.eg</t>
+          <t>160715@med.asu.edu.eg, 2025/2026</t>
         </is>
       </c>
       <c r="H195" s="5" t="inlineStr">
@@ -11477,7 +11477,7 @@
       </c>
       <c r="G235" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 160715@med.asu.edu.eg</t>
+          <t>160715@med.asu.edu.eg, 2025/2026</t>
         </is>
       </c>
       <c r="H235" s="5" t="inlineStr">
@@ -12420,45 +12420,49 @@
       </c>
     </row>
     <row r="256">
-      <c r="A256" s="2" t="inlineStr">
-        <is>
-          <t>Year 5</t>
-        </is>
-      </c>
-      <c r="B256" s="2" t="inlineStr">
+      <c r="A256" s="5" t="inlineStr">
+        <is>
+          <t>Year 5</t>
+        </is>
+      </c>
+      <c r="B256" s="5" t="inlineStr">
         <is>
           <t>A2D1</t>
         </is>
       </c>
-      <c r="C256" s="2" t="inlineStr">
+      <c r="C256" s="5" t="inlineStr">
         <is>
           <t>GASTROENTEROLOGY</t>
         </is>
       </c>
-      <c r="D256" s="2" t="inlineStr">
+      <c r="D256" s="5" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="E256" s="2" t="inlineStr">
+      <c r="E256" s="5" t="inlineStr">
         <is>
           <t>23/06/2026</t>
         </is>
       </c>
-      <c r="F256" s="2" t="inlineStr">
-        <is>
-          <t>09:00:00</t>
-        </is>
-      </c>
-      <c r="G256" s="2" t="inlineStr"/>
-      <c r="H256" s="2" t="inlineStr">
-        <is>
-          <t>0/34</t>
-        </is>
-      </c>
-      <c r="I256" s="2" t="inlineStr">
-        <is>
-          <t>Not Recorded</t>
+      <c r="F256" s="5" t="inlineStr">
+        <is>
+          <t>09:00:00</t>
+        </is>
+      </c>
+      <c r="G256" s="5" t="inlineStr">
+        <is>
+          <t>2026/2027</t>
+        </is>
+      </c>
+      <c r="H256" s="5" t="inlineStr">
+        <is>
+          <t>32/34</t>
+        </is>
+      </c>
+      <c r="I256" s="5" t="inlineStr">
+        <is>
+          <t>Recorded</t>
         </is>
       </c>
     </row>
@@ -14224,45 +14228,49 @@
       </c>
     </row>
     <row r="296">
-      <c r="A296" s="2" t="inlineStr">
-        <is>
-          <t>Year 5</t>
-        </is>
-      </c>
-      <c r="B296" s="2" t="inlineStr">
+      <c r="A296" s="5" t="inlineStr">
+        <is>
+          <t>Year 5</t>
+        </is>
+      </c>
+      <c r="B296" s="5" t="inlineStr">
         <is>
           <t>A2D2</t>
         </is>
       </c>
-      <c r="C296" s="2" t="inlineStr">
+      <c r="C296" s="5" t="inlineStr">
         <is>
           <t>GASTROENTEROLOGY</t>
         </is>
       </c>
-      <c r="D296" s="2" t="inlineStr">
+      <c r="D296" s="5" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="E296" s="2" t="inlineStr">
+      <c r="E296" s="5" t="inlineStr">
         <is>
           <t>23/06/2026</t>
         </is>
       </c>
-      <c r="F296" s="2" t="inlineStr">
-        <is>
-          <t>09:00:00</t>
-        </is>
-      </c>
-      <c r="G296" s="2" t="inlineStr"/>
-      <c r="H296" s="2" t="inlineStr">
-        <is>
-          <t>0/40</t>
-        </is>
-      </c>
-      <c r="I296" s="2" t="inlineStr">
-        <is>
-          <t>Not Recorded</t>
+      <c r="F296" s="5" t="inlineStr">
+        <is>
+          <t>09:00:00</t>
+        </is>
+      </c>
+      <c r="G296" s="5" t="inlineStr">
+        <is>
+          <t>2026/2027</t>
+        </is>
+      </c>
+      <c r="H296" s="5" t="inlineStr">
+        <is>
+          <t>7/40</t>
+        </is>
+      </c>
+      <c r="I296" s="5" t="inlineStr">
+        <is>
+          <t>Recorded</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-06-24 02:42:44
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -9677,7 +9677,7 @@
       </c>
       <c r="G195" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 160715@med.asu.edu.eg</t>
+          <t>160715@med.asu.edu.eg, 2025/2026</t>
         </is>
       </c>
       <c r="H195" s="5" t="inlineStr">
@@ -11477,7 +11477,7 @@
       </c>
       <c r="G235" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 160715@med.asu.edu.eg</t>
+          <t>160715@med.asu.edu.eg, 2025/2026</t>
         </is>
       </c>
       <c r="H235" s="5" t="inlineStr">
@@ -13066,7 +13066,7 @@
       </c>
       <c r="G270" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2027/2028</t>
+          <t>2027/2028, 2025/2026</t>
         </is>
       </c>
       <c r="H270" s="5" t="inlineStr">
@@ -13113,7 +13113,7 @@
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2027/2028, 2026/2027</t>
+          <t>2027/2028, 2025/2026, 2026/2027</t>
         </is>
       </c>
       <c r="H271" s="5" t="inlineStr">
@@ -14874,7 +14874,7 @@
       </c>
       <c r="G310" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2027/2028</t>
+          <t>2027/2028, 2025/2026</t>
         </is>
       </c>
       <c r="H310" s="5" t="inlineStr">
@@ -14921,7 +14921,7 @@
       </c>
       <c r="G311" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2027/2028, 2026/2027</t>
+          <t>2027/2028, 2025/2026, 2026/2027</t>
         </is>
       </c>
       <c r="H311" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-06-25 17:07:08
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -13094,7 +13094,7 @@
       </c>
       <c r="G270" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2025/2026</t>
+          <t>2025/2026, 2027/2028</t>
         </is>
       </c>
       <c r="H270" s="5" t="inlineStr">
@@ -13141,7 +13141,7 @@
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2025/2026, 2026/2027</t>
+          <t>2025/2026, 2026/2027, 2027/2028</t>
         </is>
       </c>
       <c r="H271" s="5" t="inlineStr">
@@ -14906,7 +14906,7 @@
       </c>
       <c r="G310" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2025/2026</t>
+          <t>2025/2026, 2027/2028</t>
         </is>
       </c>
       <c r="H310" s="5" t="inlineStr">
@@ -14953,7 +14953,7 @@
       </c>
       <c r="G311" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2025/2026, 2026/2027</t>
+          <t>2025/2026, 2026/2027, 2027/2028</t>
         </is>
       </c>
       <c r="H311" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-06-26 22:07:08
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -13094,7 +13094,7 @@
       </c>
       <c r="G270" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2027/2028</t>
+          <t>2027/2028, 2025/2026</t>
         </is>
       </c>
       <c r="H270" s="5" t="inlineStr">
@@ -13141,7 +13141,7 @@
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>2026/2027, 2025/2026, 2027/2028</t>
+          <t>2027/2028, 2026/2027, 2025/2026</t>
         </is>
       </c>
       <c r="H271" s="5" t="inlineStr">
@@ -14906,7 +14906,7 @@
       </c>
       <c r="G310" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2027/2028</t>
+          <t>2027/2028, 2025/2026</t>
         </is>
       </c>
       <c r="H310" s="5" t="inlineStr">
@@ -14953,7 +14953,7 @@
       </c>
       <c r="G311" s="5" t="inlineStr">
         <is>
-          <t>2026/2027, 2025/2026, 2027/2028</t>
+          <t>2027/2028, 2026/2027, 2025/2026</t>
         </is>
       </c>
       <c r="H311" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-06-28 21:58:19
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -9737,7 +9737,7 @@
       </c>
       <c r="G195" s="5" t="inlineStr">
         <is>
-          <t>160715@med.asu.edu.eg, 2025/2026</t>
+          <t>2025/2026, 160715@med.asu.edu.eg</t>
         </is>
       </c>
       <c r="H195" s="5" t="inlineStr">
@@ -11549,7 +11549,7 @@
       </c>
       <c r="G235" s="5" t="inlineStr">
         <is>
-          <t>160715@med.asu.edu.eg, 2025/2026</t>
+          <t>2025/2026, 160715@med.asu.edu.eg</t>
         </is>
       </c>
       <c r="H235" s="5" t="inlineStr">
@@ -13142,7 +13142,7 @@
       </c>
       <c r="G270" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2027/2028</t>
+          <t>2027/2028, 2025/2026</t>
         </is>
       </c>
       <c r="H270" s="5" t="inlineStr">
@@ -13189,7 +13189,7 @@
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>2026/2027, 2025/2026, 2027/2028</t>
+          <t>2026/2027, 2027/2028, 2025/2026</t>
         </is>
       </c>
       <c r="H271" s="5" t="inlineStr">
@@ -14958,7 +14958,7 @@
       </c>
       <c r="G310" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2027/2028</t>
+          <t>2027/2028, 2025/2026</t>
         </is>
       </c>
       <c r="H310" s="5" t="inlineStr">
@@ -15005,7 +15005,7 @@
       </c>
       <c r="G311" s="5" t="inlineStr">
         <is>
-          <t>2026/2027, 2025/2026, 2027/2028</t>
+          <t>2026/2027, 2027/2028, 2025/2026</t>
         </is>
       </c>
       <c r="H311" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-06-29 19:00:46
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -9757,7 +9757,7 @@
       </c>
       <c r="G195" s="5" t="inlineStr">
         <is>
-          <t>160715@med.asu.edu.eg, 2025/2026</t>
+          <t>2025/2026, 160715@med.asu.edu.eg</t>
         </is>
       </c>
       <c r="H195" s="5" t="inlineStr">
@@ -11573,7 +11573,7 @@
       </c>
       <c r="G235" s="5" t="inlineStr">
         <is>
-          <t>160715@med.asu.edu.eg, 2025/2026</t>
+          <t>2025/2026, 160715@med.asu.edu.eg</t>
         </is>
       </c>
       <c r="H235" s="5" t="inlineStr">
@@ -13213,7 +13213,7 @@
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>2026/2027, 2025/2026, 2027/2028</t>
+          <t>2025/2026, 2026/2027, 2027/2028</t>
         </is>
       </c>
       <c r="H271" s="5" t="inlineStr">
@@ -15029,7 +15029,7 @@
       </c>
       <c r="G311" s="5" t="inlineStr">
         <is>
-          <t>2026/2027, 2025/2026, 2027/2028</t>
+          <t>2025/2026, 2026/2027, 2027/2028</t>
         </is>
       </c>
       <c r="H311" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-06-30 16:20:39
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -13233,7 +13233,7 @@
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>2026/2027, 2027/2028, 2025/2026</t>
+          <t>2027/2028, 2025/2026, 2026/2027</t>
         </is>
       </c>
       <c r="H271" s="5" t="inlineStr">
@@ -15057,7 +15057,7 @@
       </c>
       <c r="G311" s="5" t="inlineStr">
         <is>
-          <t>2026/2027, 2027/2028, 2025/2026</t>
+          <t>2027/2028, 2025/2026, 2026/2027</t>
         </is>
       </c>
       <c r="H311" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-07-01 17:49:33
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -13206,7 +13206,7 @@
       </c>
       <c r="G270" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2025/2026</t>
+          <t>2025/2026, 2027/2028</t>
         </is>
       </c>
       <c r="H270" s="5" t="inlineStr">
@@ -13253,7 +13253,7 @@
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2025/2026, 2026/2027</t>
+          <t>2025/2026, 2026/2027, 2027/2028</t>
         </is>
       </c>
       <c r="H271" s="5" t="inlineStr">
@@ -15034,7 +15034,7 @@
       </c>
       <c r="G310" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2025/2026</t>
+          <t>2025/2026, 2027/2028</t>
         </is>
       </c>
       <c r="H310" s="5" t="inlineStr">
@@ -15081,7 +15081,7 @@
       </c>
       <c r="G311" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2025/2026, 2026/2027</t>
+          <t>2025/2026, 2026/2027, 2027/2028</t>
         </is>
       </c>
       <c r="H311" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-07-04 22:52:41
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -9805,7 +9805,7 @@
       </c>
       <c r="G195" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 160715@med.asu.edu.eg</t>
+          <t>160715@med.asu.edu.eg, 2025/2026</t>
         </is>
       </c>
       <c r="H195" s="5" t="inlineStr">
@@ -11625,7 +11625,7 @@
       </c>
       <c r="G235" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 160715@med.asu.edu.eg</t>
+          <t>160715@med.asu.edu.eg, 2025/2026</t>
         </is>
       </c>
       <c r="H235" s="5" t="inlineStr">
@@ -13277,7 +13277,7 @@
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2025/2026, 2026/2027</t>
+          <t>2026/2027, 2027/2028, 2025/2026</t>
         </is>
       </c>
       <c r="H271" s="5" t="inlineStr">
@@ -15109,7 +15109,7 @@
       </c>
       <c r="G311" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2025/2026, 2026/2027</t>
+          <t>2026/2027, 2027/2028, 2025/2026</t>
         </is>
       </c>
       <c r="H311" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-07-09 04:46:05
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -9869,7 +9869,7 @@
       </c>
       <c r="G195" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 160715@med.asu.edu.eg</t>
+          <t>160715@med.asu.edu.eg, 2025/2026</t>
         </is>
       </c>
       <c r="H195" s="5" t="inlineStr">
@@ -11697,7 +11697,7 @@
       </c>
       <c r="G235" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 160715@med.asu.edu.eg</t>
+          <t>160715@med.asu.edu.eg, 2025/2026</t>
         </is>
       </c>
       <c r="H235" s="5" t="inlineStr">
@@ -13302,7 +13302,7 @@
       </c>
       <c r="G270" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2025/2026</t>
+          <t>2025/2026, 2027/2028</t>
         </is>
       </c>
       <c r="H270" s="5" t="inlineStr">
@@ -13349,7 +13349,7 @@
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>2026/2027, 2027/2028, 2025/2026</t>
+          <t>2026/2027, 2025/2026, 2027/2028</t>
         </is>
       </c>
       <c r="H271" s="5" t="inlineStr">
@@ -15150,7 +15150,7 @@
       </c>
       <c r="G310" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2025/2026</t>
+          <t>2025/2026, 2027/2028</t>
         </is>
       </c>
       <c r="H310" s="5" t="inlineStr">
@@ -15197,7 +15197,7 @@
       </c>
       <c r="G311" s="5" t="inlineStr">
         <is>
-          <t>2026/2027, 2027/2028, 2025/2026</t>
+          <t>2026/2027, 2025/2026, 2027/2028</t>
         </is>
       </c>
       <c r="H311" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-07-09 14:44:04
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -9869,7 +9869,7 @@
       </c>
       <c r="G195" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 160715@med.asu.edu.eg</t>
+          <t>160715@med.asu.edu.eg, 2025/2026</t>
         </is>
       </c>
       <c r="H195" s="5" t="inlineStr">
@@ -11697,7 +11697,7 @@
       </c>
       <c r="G235" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 160715@med.asu.edu.eg</t>
+          <t>160715@med.asu.edu.eg, 2025/2026</t>
         </is>
       </c>
       <c r="H235" s="5" t="inlineStr">
@@ -13302,7 +13302,7 @@
       </c>
       <c r="G270" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2025/2026</t>
+          <t>2025/2026, 2027/2028</t>
         </is>
       </c>
       <c r="H270" s="5" t="inlineStr">
@@ -13349,7 +13349,7 @@
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2025/2026, 2026/2027</t>
+          <t>2026/2027, 2025/2026, 2027/2028</t>
         </is>
       </c>
       <c r="H271" s="5" t="inlineStr">
@@ -15150,7 +15150,7 @@
       </c>
       <c r="G310" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2025/2026</t>
+          <t>2025/2026, 2027/2028</t>
         </is>
       </c>
       <c r="H310" s="5" t="inlineStr">
@@ -15197,7 +15197,7 @@
       </c>
       <c r="G311" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2025/2026, 2026/2027</t>
+          <t>2026/2027, 2025/2026, 2027/2028</t>
         </is>
       </c>
       <c r="H311" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-07-09 19:28:55
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -13302,7 +13302,7 @@
       </c>
       <c r="G270" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2025/2026</t>
+          <t>2025/2026, 2027/2028</t>
         </is>
       </c>
       <c r="H270" s="5" t="inlineStr">
@@ -13349,7 +13349,7 @@
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>2026/2027, 2027/2028, 2025/2026</t>
+          <t>2026/2027, 2025/2026, 2027/2028</t>
         </is>
       </c>
       <c r="H271" s="5" t="inlineStr">
@@ -15150,7 +15150,7 @@
       </c>
       <c r="G310" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2025/2026</t>
+          <t>2025/2026, 2027/2028</t>
         </is>
       </c>
       <c r="H310" s="5" t="inlineStr">
@@ -15197,7 +15197,7 @@
       </c>
       <c r="G311" s="5" t="inlineStr">
         <is>
-          <t>2026/2027, 2027/2028, 2025/2026</t>
+          <t>2026/2027, 2025/2026, 2027/2028</t>
         </is>
       </c>
       <c r="H311" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-07-10 10:18:53
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -9869,7 +9869,7 @@
       </c>
       <c r="G195" s="5" t="inlineStr">
         <is>
-          <t>160715@med.asu.edu.eg, 2025/2026</t>
+          <t>2025/2026, 160715@med.asu.edu.eg</t>
         </is>
       </c>
       <c r="H195" s="5" t="inlineStr">
@@ -11697,7 +11697,7 @@
       </c>
       <c r="G235" s="5" t="inlineStr">
         <is>
-          <t>160715@med.asu.edu.eg, 2025/2026</t>
+          <t>2025/2026, 160715@med.asu.edu.eg</t>
         </is>
       </c>
       <c r="H235" s="5" t="inlineStr">
@@ -13349,7 +13349,7 @@
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2027/2028, 2026/2027</t>
+          <t>2025/2026, 2026/2027, 2027/2028</t>
         </is>
       </c>
       <c r="H271" s="5" t="inlineStr">
@@ -15197,7 +15197,7 @@
       </c>
       <c r="G311" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2027/2028, 2026/2027</t>
+          <t>2025/2026, 2026/2027, 2027/2028</t>
         </is>
       </c>
       <c r="H311" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-07-11 02:04:46
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -13349,7 +13349,7 @@
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2027/2028, 2026/2027</t>
+          <t>2025/2026, 2026/2027, 2027/2028</t>
         </is>
       </c>
       <c r="H271" s="5" t="inlineStr">
@@ -15197,7 +15197,7 @@
       </c>
       <c r="G311" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2027/2028, 2026/2027</t>
+          <t>2025/2026, 2026/2027, 2027/2028</t>
         </is>
       </c>
       <c r="H311" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-07-11 13:05:23
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -1021,7 +1021,7 @@
       </c>
       <c r="L10" s="4" t="inlineStr">
         <is>
-          <t>77.9%</t>
+          <t>78.1%</t>
         </is>
       </c>
     </row>
@@ -1739,7 +1739,7 @@
       </c>
       <c r="S20" s="4" t="inlineStr">
         <is>
-          <t>79.3%</t>
+          <t>80.9%</t>
         </is>
       </c>
     </row>
@@ -9889,7 +9889,7 @@
       </c>
       <c r="G195" s="5" t="inlineStr">
         <is>
-          <t>160715@med.asu.edu.eg, 2025/2026</t>
+          <t>2025/2026, 160715@med.asu.edu.eg</t>
         </is>
       </c>
       <c r="H195" s="5" t="inlineStr">
@@ -10951,7 +10951,7 @@
       </c>
       <c r="H218" s="5" t="inlineStr">
         <is>
-          <t>19/37</t>
+          <t>34/37</t>
         </is>
       </c>
       <c r="I218" s="5" t="inlineStr">
@@ -11721,7 +11721,7 @@
       </c>
       <c r="G235" s="5" t="inlineStr">
         <is>
-          <t>160715@med.asu.edu.eg, 2025/2026</t>
+          <t>2025/2026, 160715@med.asu.edu.eg</t>
         </is>
       </c>
       <c r="H235" s="5" t="inlineStr">
@@ -13330,7 +13330,7 @@
       </c>
       <c r="G270" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2027/2028</t>
+          <t>2027/2028, 2025/2026</t>
         </is>
       </c>
       <c r="H270" s="5" t="inlineStr">
@@ -13377,7 +13377,7 @@
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2027/2028, 2026/2027</t>
+          <t>2027/2028, 2025/2026, 2026/2027</t>
         </is>
       </c>
       <c r="H271" s="5" t="inlineStr">
@@ -15178,7 +15178,7 @@
       </c>
       <c r="G310" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2027/2028</t>
+          <t>2027/2028, 2025/2026</t>
         </is>
       </c>
       <c r="H310" s="5" t="inlineStr">
@@ -15225,7 +15225,7 @@
       </c>
       <c r="G311" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2027/2028, 2026/2027</t>
+          <t>2027/2028, 2025/2026, 2026/2027</t>
         </is>
       </c>
       <c r="H311" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-07-11 15:49:39
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -9114,7 +9114,7 @@
       </c>
       <c r="G178" s="5" t="inlineStr">
         <is>
-          <t>2025/2026</t>
+          <t>2026/2027, 2025/2026</t>
         </is>
       </c>
       <c r="H178" s="5" t="inlineStr">
@@ -10946,7 +10946,7 @@
       </c>
       <c r="G218" s="5" t="inlineStr">
         <is>
-          <t>2025/2026</t>
+          <t>2026/2027, 2025/2026</t>
         </is>
       </c>
       <c r="H218" s="5" t="inlineStr">
@@ -13330,7 +13330,7 @@
       </c>
       <c r="G270" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2025/2026</t>
+          <t>2025/2026, 2027/2028</t>
         </is>
       </c>
       <c r="H270" s="5" t="inlineStr">
@@ -13377,7 +13377,7 @@
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2026/2027, 2025/2026</t>
+          <t>2026/2027, 2025/2026, 2027/2028</t>
         </is>
       </c>
       <c r="H271" s="5" t="inlineStr">
@@ -15178,7 +15178,7 @@
       </c>
       <c r="G310" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2025/2026</t>
+          <t>2025/2026, 2027/2028</t>
         </is>
       </c>
       <c r="H310" s="5" t="inlineStr">
@@ -15225,7 +15225,7 @@
       </c>
       <c r="G311" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2026/2027, 2025/2026</t>
+          <t>2026/2027, 2025/2026, 2027/2028</t>
         </is>
       </c>
       <c r="H311" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-07-12 10:21:43
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -802,7 +802,7 @@
         </is>
       </c>
       <c r="L6" s="4" t="n">
-        <v>230</v>
+        <v>232</v>
       </c>
     </row>
     <row r="7">
@@ -853,7 +853,7 @@
         </is>
       </c>
       <c r="L7" s="4" t="n">
-        <v>67</v>
+        <v>65</v>
       </c>
     </row>
     <row r="8">
@@ -964,7 +964,7 @@
       </c>
       <c r="L9" s="4" t="inlineStr">
         <is>
-          <t>71.7%</t>
+          <t>72.3%</t>
         </is>
       </c>
     </row>
@@ -1021,7 +1021,7 @@
       </c>
       <c r="L10" s="4" t="inlineStr">
         <is>
-          <t>78.1%</t>
+          <t>78.2%</t>
         </is>
       </c>
     </row>
@@ -1318,22 +1318,22 @@
         <v>40</v>
       </c>
       <c r="O15" s="4" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="P15" s="4" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="Q15" s="4" t="n">
         <v>3</v>
       </c>
       <c r="R15" s="4" t="inlineStr">
         <is>
-          <t>70.0%</t>
+          <t>72.5%</t>
         </is>
       </c>
       <c r="S15" s="4" t="inlineStr">
         <is>
-          <t>78.6%</t>
+          <t>78.5%</t>
         </is>
       </c>
     </row>
@@ -1400,22 +1400,22 @@
         <v>41</v>
       </c>
       <c r="O16" s="4" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="P16" s="4" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="Q16" s="4" t="n">
         <v>3</v>
       </c>
       <c r="R16" s="4" t="inlineStr">
         <is>
-          <t>63.4%</t>
+          <t>65.9%</t>
         </is>
       </c>
       <c r="S16" s="4" t="inlineStr">
         <is>
-          <t>79.5%</t>
+          <t>79.8%</t>
         </is>
       </c>
     </row>
@@ -2396,45 +2396,49 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="2" t="inlineStr">
-        <is>
-          <t>Year 5</t>
-        </is>
-      </c>
-      <c r="B32" s="2" t="inlineStr">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>Year 5</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="inlineStr">
         <is>
           <t>A2A1</t>
         </is>
       </c>
-      <c r="C32" s="2" t="inlineStr">
+      <c r="C32" s="5" t="inlineStr">
         <is>
           <t>NEUROLOGY</t>
         </is>
       </c>
-      <c r="D32" s="2" t="inlineStr">
+      <c r="D32" s="5" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="E32" s="2" t="inlineStr">
+      <c r="E32" s="5" t="inlineStr">
         <is>
           <t>12/07/2026</t>
         </is>
       </c>
-      <c r="F32" s="2" t="inlineStr">
-        <is>
-          <t>09:00:00</t>
-        </is>
-      </c>
-      <c r="G32" s="2" t="inlineStr"/>
-      <c r="H32" s="2" t="inlineStr">
-        <is>
-          <t>0/37</t>
-        </is>
-      </c>
-      <c r="I32" s="2" t="inlineStr">
-        <is>
-          <t>Not Recorded</t>
+      <c r="F32" s="5" t="inlineStr">
+        <is>
+          <t>09:00:00</t>
+        </is>
+      </c>
+      <c r="G32" s="5" t="inlineStr">
+        <is>
+          <t>2025/2026</t>
+        </is>
+      </c>
+      <c r="H32" s="5" t="inlineStr">
+        <is>
+          <t>28/37</t>
+        </is>
+      </c>
+      <c r="I32" s="5" t="inlineStr">
+        <is>
+          <t>Recorded</t>
         </is>
       </c>
     </row>
@@ -4259,45 +4263,49 @@
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="2" t="inlineStr">
-        <is>
-          <t>Year 5</t>
-        </is>
-      </c>
-      <c r="B73" s="2" t="inlineStr">
+      <c r="A73" s="5" t="inlineStr">
+        <is>
+          <t>Year 5</t>
+        </is>
+      </c>
+      <c r="B73" s="5" t="inlineStr">
         <is>
           <t>A2A2</t>
         </is>
       </c>
-      <c r="C73" s="2" t="inlineStr">
+      <c r="C73" s="5" t="inlineStr">
         <is>
           <t>NEUROLOGY</t>
         </is>
       </c>
-      <c r="D73" s="2" t="inlineStr">
+      <c r="D73" s="5" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="E73" s="2" t="inlineStr">
+      <c r="E73" s="5" t="inlineStr">
         <is>
           <t>12/07/2026</t>
         </is>
       </c>
-      <c r="F73" s="2" t="inlineStr">
-        <is>
-          <t>09:00:00</t>
-        </is>
-      </c>
-      <c r="G73" s="2" t="inlineStr"/>
-      <c r="H73" s="2" t="inlineStr">
-        <is>
-          <t>0/35</t>
-        </is>
-      </c>
-      <c r="I73" s="2" t="inlineStr">
-        <is>
-          <t>Not Recorded</t>
+      <c r="F73" s="5" t="inlineStr">
+        <is>
+          <t>09:00:00</t>
+        </is>
+      </c>
+      <c r="G73" s="5" t="inlineStr">
+        <is>
+          <t>2025/2026</t>
+        </is>
+      </c>
+      <c r="H73" s="5" t="inlineStr">
+        <is>
+          <t>31/35</t>
+        </is>
+      </c>
+      <c r="I73" s="5" t="inlineStr">
+        <is>
+          <t>Recorded</t>
         </is>
       </c>
     </row>
@@ -9889,7 +9897,7 @@
       </c>
       <c r="G195" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 160715@med.asu.edu.eg</t>
+          <t>160715@med.asu.edu.eg, 2025/2026</t>
         </is>
       </c>
       <c r="H195" s="5" t="inlineStr">
@@ -11721,7 +11729,7 @@
       </c>
       <c r="G235" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 160715@med.asu.edu.eg</t>
+          <t>160715@med.asu.edu.eg, 2025/2026</t>
         </is>
       </c>
       <c r="H235" s="5" t="inlineStr">
@@ -13377,7 +13385,7 @@
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2027/2028, 2026/2027</t>
+          <t>2025/2026, 2026/2027, 2027/2028</t>
         </is>
       </c>
       <c r="H271" s="5" t="inlineStr">
@@ -15225,7 +15233,7 @@
       </c>
       <c r="G311" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2027/2028, 2026/2027</t>
+          <t>2025/2026, 2026/2027, 2027/2028</t>
         </is>
       </c>
       <c r="H311" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-07-12 15:54:00
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -13358,7 +13358,7 @@
       </c>
       <c r="G270" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2027/2028</t>
+          <t>2027/2028, 2025/2026</t>
         </is>
       </c>
       <c r="H270" s="5" t="inlineStr">
@@ -13405,7 +13405,7 @@
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2026/2027, 2027/2028</t>
+          <t>2027/2028, 2025/2026, 2026/2027</t>
         </is>
       </c>
       <c r="H271" s="5" t="inlineStr">
@@ -15206,7 +15206,7 @@
       </c>
       <c r="G310" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2027/2028</t>
+          <t>2027/2028, 2025/2026</t>
         </is>
       </c>
       <c r="H310" s="5" t="inlineStr">
@@ -15253,7 +15253,7 @@
       </c>
       <c r="G311" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2026/2027, 2027/2028</t>
+          <t>2027/2028, 2025/2026, 2026/2027</t>
         </is>
       </c>
       <c r="H311" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-07-12 16:53:12
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -13358,7 +13358,7 @@
       </c>
       <c r="G270" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2025/2026</t>
+          <t>2025/2026, 2027/2028</t>
         </is>
       </c>
       <c r="H270" s="5" t="inlineStr">
@@ -13405,7 +13405,7 @@
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2025/2026, 2026/2027</t>
+          <t>2025/2026, 2026/2027, 2027/2028</t>
         </is>
       </c>
       <c r="H271" s="5" t="inlineStr">
@@ -15206,7 +15206,7 @@
       </c>
       <c r="G310" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2025/2026</t>
+          <t>2025/2026, 2027/2028</t>
         </is>
       </c>
       <c r="H310" s="5" t="inlineStr">
@@ -15253,7 +15253,7 @@
       </c>
       <c r="G311" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2025/2026, 2026/2027</t>
+          <t>2025/2026, 2026/2027, 2027/2028</t>
         </is>
       </c>
       <c r="H311" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-07-12 20:05:32
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -9909,7 +9909,7 @@
       </c>
       <c r="G195" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 160715@med.asu.edu.eg</t>
+          <t>160715@med.asu.edu.eg, 2025/2026</t>
         </is>
       </c>
       <c r="H195" s="5" t="inlineStr">
@@ -11745,7 +11745,7 @@
       </c>
       <c r="G235" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 160715@med.asu.edu.eg</t>
+          <t>160715@med.asu.edu.eg, 2025/2026</t>
         </is>
       </c>
       <c r="H235" s="5" t="inlineStr">
@@ -13405,7 +13405,7 @@
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2027/2028, 2026/2027</t>
+          <t>2025/2026, 2026/2027, 2027/2028</t>
         </is>
       </c>
       <c r="H271" s="5" t="inlineStr">
@@ -15253,7 +15253,7 @@
       </c>
       <c r="G311" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2027/2028, 2026/2027</t>
+          <t>2025/2026, 2026/2027, 2027/2028</t>
         </is>
       </c>
       <c r="H311" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-07-12 21:42:39
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -9909,7 +9909,7 @@
       </c>
       <c r="G195" s="5" t="inlineStr">
         <is>
-          <t>160715@med.asu.edu.eg, 2025/2026</t>
+          <t>2025/2026, 160715@med.asu.edu.eg</t>
         </is>
       </c>
       <c r="H195" s="5" t="inlineStr">
@@ -11745,7 +11745,7 @@
       </c>
       <c r="G235" s="5" t="inlineStr">
         <is>
-          <t>160715@med.asu.edu.eg, 2025/2026</t>
+          <t>2025/2026, 160715@med.asu.edu.eg</t>
         </is>
       </c>
       <c r="H235" s="5" t="inlineStr">
@@ -13358,7 +13358,7 @@
       </c>
       <c r="G270" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2027/2028</t>
+          <t>2027/2028, 2025/2026</t>
         </is>
       </c>
       <c r="H270" s="5" t="inlineStr">
@@ -13405,7 +13405,7 @@
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2026/2027, 2027/2028</t>
+          <t>2027/2028, 2025/2026, 2026/2027</t>
         </is>
       </c>
       <c r="H271" s="5" t="inlineStr">
@@ -15206,7 +15206,7 @@
       </c>
       <c r="G310" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2027/2028</t>
+          <t>2027/2028, 2025/2026</t>
         </is>
       </c>
       <c r="H310" s="5" t="inlineStr">
@@ -15253,7 +15253,7 @@
       </c>
       <c r="G311" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2026/2027, 2027/2028</t>
+          <t>2027/2028, 2025/2026, 2026/2027</t>
         </is>
       </c>
       <c r="H311" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-07-13 18:28:38
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -9937,7 +9937,7 @@
       </c>
       <c r="G195" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 160715@med.asu.edu.eg</t>
+          <t>160715@med.asu.edu.eg, 2025/2026</t>
         </is>
       </c>
       <c r="H195" s="5" t="inlineStr">
@@ -11777,7 +11777,7 @@
       </c>
       <c r="G235" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 160715@med.asu.edu.eg</t>
+          <t>160715@med.asu.edu.eg, 2025/2026</t>
         </is>
       </c>
       <c r="H235" s="5" t="inlineStr">
@@ -13394,7 +13394,7 @@
       </c>
       <c r="G270" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2027/2028</t>
+          <t>2027/2028, 2025/2026</t>
         </is>
       </c>
       <c r="H270" s="5" t="inlineStr">
@@ -13441,7 +13441,7 @@
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2026/2027, 2027/2028</t>
+          <t>2027/2028, 2025/2026, 2026/2027</t>
         </is>
       </c>
       <c r="H271" s="5" t="inlineStr">
@@ -15242,7 +15242,7 @@
       </c>
       <c r="G310" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2027/2028</t>
+          <t>2027/2028, 2025/2026</t>
         </is>
       </c>
       <c r="H310" s="5" t="inlineStr">
@@ -15289,7 +15289,7 @@
       </c>
       <c r="G311" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2026/2027, 2027/2028</t>
+          <t>2027/2028, 2025/2026, 2026/2027</t>
         </is>
       </c>
       <c r="H311" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-07-14 15:19:41
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -9957,7 +9957,7 @@
       </c>
       <c r="G195" s="5" t="inlineStr">
         <is>
-          <t>160715@med.asu.edu.eg, 2025/2026</t>
+          <t>2025/2026, 160715@med.asu.edu.eg</t>
         </is>
       </c>
       <c r="H195" s="5" t="inlineStr">
@@ -11801,7 +11801,7 @@
       </c>
       <c r="G235" s="5" t="inlineStr">
         <is>
-          <t>160715@med.asu.edu.eg, 2025/2026</t>
+          <t>2025/2026, 160715@med.asu.edu.eg</t>
         </is>
       </c>
       <c r="H235" s="5" t="inlineStr">
@@ -13465,7 +13465,7 @@
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>2026/2027, 2027/2028, 2025/2026</t>
+          <t>2027/2028, 2026/2027, 2025/2026</t>
         </is>
       </c>
       <c r="H271" s="5" t="inlineStr">
@@ -15313,7 +15313,7 @@
       </c>
       <c r="G311" s="5" t="inlineStr">
         <is>
-          <t>2026/2027, 2027/2028, 2025/2026</t>
+          <t>2027/2028, 2026/2027, 2025/2026</t>
         </is>
       </c>
       <c r="H311" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-07-15 15:22:23
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -9966,7 +9966,7 @@
       </c>
       <c r="G195" s="5" t="inlineStr">
         <is>
-          <t>160715@med.asu.edu.eg, 2025/2026</t>
+          <t>2025/2026, 160715@med.asu.edu.eg</t>
         </is>
       </c>
       <c r="H195" s="5" t="inlineStr">
@@ -11814,7 +11814,7 @@
       </c>
       <c r="G235" s="5" t="inlineStr">
         <is>
-          <t>160715@med.asu.edu.eg, 2025/2026</t>
+          <t>2025/2026, 160715@med.asu.edu.eg</t>
         </is>
       </c>
       <c r="H235" s="5" t="inlineStr">
@@ -13482,7 +13482,7 @@
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2027/2028, 2026/2027</t>
+          <t>2025/2026, 2026/2027, 2027/2028</t>
         </is>
       </c>
       <c r="H271" s="5" t="inlineStr">
@@ -15330,7 +15330,7 @@
       </c>
       <c r="G311" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2027/2028, 2026/2027</t>
+          <t>2025/2026, 2026/2027, 2027/2028</t>
         </is>
       </c>
       <c r="H311" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-07-15 19:01:42
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -9966,7 +9966,7 @@
       </c>
       <c r="G195" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 160715@med.asu.edu.eg</t>
+          <t>160715@med.asu.edu.eg, 2025/2026</t>
         </is>
       </c>
       <c r="H195" s="5" t="inlineStr">
@@ -11814,7 +11814,7 @@
       </c>
       <c r="G235" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 160715@med.asu.edu.eg</t>
+          <t>160715@med.asu.edu.eg, 2025/2026</t>
         </is>
       </c>
       <c r="H235" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-07-17 07:59:23
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -13443,7 +13443,7 @@
       </c>
       <c r="G270" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2027/2028</t>
+          <t>2027/2028, 2025/2026</t>
         </is>
       </c>
       <c r="H270" s="5" t="inlineStr">
@@ -13490,7 +13490,7 @@
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2027/2028, 2026/2027</t>
+          <t>2027/2028, 2025/2026, 2026/2027</t>
         </is>
       </c>
       <c r="H271" s="5" t="inlineStr">
@@ -15291,7 +15291,7 @@
       </c>
       <c r="G310" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2027/2028</t>
+          <t>2027/2028, 2025/2026</t>
         </is>
       </c>
       <c r="H310" s="5" t="inlineStr">
@@ -15338,7 +15338,7 @@
       </c>
       <c r="G311" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2027/2028, 2026/2027</t>
+          <t>2027/2028, 2025/2026, 2026/2027</t>
         </is>
       </c>
       <c r="H311" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-07-17 10:02:08
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -13443,7 +13443,7 @@
       </c>
       <c r="G270" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2025/2026</t>
+          <t>2025/2026, 2027/2028</t>
         </is>
       </c>
       <c r="H270" s="5" t="inlineStr">
@@ -13490,7 +13490,7 @@
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2025/2026, 2026/2027</t>
+          <t>2025/2026, 2027/2028, 2026/2027</t>
         </is>
       </c>
       <c r="H271" s="5" t="inlineStr">
@@ -15291,7 +15291,7 @@
       </c>
       <c r="G310" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2025/2026</t>
+          <t>2025/2026, 2027/2028</t>
         </is>
       </c>
       <c r="H310" s="5" t="inlineStr">
@@ -15338,7 +15338,7 @@
       </c>
       <c r="G311" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2025/2026, 2026/2027</t>
+          <t>2025/2026, 2027/2028, 2026/2027</t>
         </is>
       </c>
       <c r="H311" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-07-18 10:14:09
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -9974,7 +9974,7 @@
       </c>
       <c r="G195" s="5" t="inlineStr">
         <is>
-          <t>160715@med.asu.edu.eg, 2025/2026</t>
+          <t>2025/2026, 160715@med.asu.edu.eg</t>
         </is>
       </c>
       <c r="H195" s="5" t="inlineStr">
@@ -11830,7 +11830,7 @@
       </c>
       <c r="G235" s="5" t="inlineStr">
         <is>
-          <t>160715@med.asu.edu.eg, 2025/2026</t>
+          <t>2025/2026, 160715@med.asu.edu.eg</t>
         </is>
       </c>
       <c r="H235" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-07-18 13:01:00
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -9974,7 +9974,7 @@
       </c>
       <c r="G195" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 160715@med.asu.edu.eg</t>
+          <t>160715@med.asu.edu.eg, 2025/2026</t>
         </is>
       </c>
       <c r="H195" s="5" t="inlineStr">
@@ -11830,7 +11830,7 @@
       </c>
       <c r="G235" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 160715@med.asu.edu.eg</t>
+          <t>160715@med.asu.edu.eg, 2025/2026</t>
         </is>
       </c>
       <c r="H235" s="5" t="inlineStr">
@@ -13498,7 +13498,7 @@
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2026/2027, 2027/2028</t>
+          <t>2025/2026, 2027/2028, 2026/2027</t>
         </is>
       </c>
       <c r="H271" s="5" t="inlineStr">
@@ -15346,7 +15346,7 @@
       </c>
       <c r="G311" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2026/2027, 2027/2028</t>
+          <t>2025/2026, 2027/2028, 2026/2027</t>
         </is>
       </c>
       <c r="H311" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-07-19 17:53:32
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -13498,7 +13498,7 @@
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2026/2027, 2025/2026</t>
+          <t>2026/2027, 2027/2028, 2025/2026</t>
         </is>
       </c>
       <c r="H271" s="5" t="inlineStr">
@@ -15346,7 +15346,7 @@
       </c>
       <c r="G311" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2026/2027, 2025/2026</t>
+          <t>2026/2027, 2027/2028, 2025/2026</t>
         </is>
       </c>
       <c r="H311" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-07-19 18:57:54
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -13498,7 +13498,7 @@
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>2026/2027, 2027/2028, 2025/2026</t>
+          <t>2027/2028, 2026/2027, 2025/2026</t>
         </is>
       </c>
       <c r="H271" s="5" t="inlineStr">
@@ -15346,7 +15346,7 @@
       </c>
       <c r="G311" s="5" t="inlineStr">
         <is>
-          <t>2026/2027, 2027/2028, 2025/2026</t>
+          <t>2027/2028, 2026/2027, 2025/2026</t>
         </is>
       </c>
       <c r="H311" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-07-19 22:44:21
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -9974,7 +9974,7 @@
       </c>
       <c r="G195" s="5" t="inlineStr">
         <is>
-          <t>160715@med.asu.edu.eg, 2025/2026</t>
+          <t>2025/2026, 160715@med.asu.edu.eg</t>
         </is>
       </c>
       <c r="H195" s="5" t="inlineStr">
@@ -11830,7 +11830,7 @@
       </c>
       <c r="G235" s="5" t="inlineStr">
         <is>
-          <t>160715@med.asu.edu.eg, 2025/2026</t>
+          <t>2025/2026, 160715@med.asu.edu.eg</t>
         </is>
       </c>
       <c r="H235" s="5" t="inlineStr">
@@ -13451,7 +13451,7 @@
       </c>
       <c r="G270" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2025/2026</t>
+          <t>2025/2026, 2027/2028</t>
         </is>
       </c>
       <c r="H270" s="5" t="inlineStr">
@@ -13498,7 +13498,7 @@
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2025/2026, 2026/2027</t>
+          <t>2025/2026, 2027/2028, 2026/2027</t>
         </is>
       </c>
       <c r="H271" s="5" t="inlineStr">
@@ -15299,7 +15299,7 @@
       </c>
       <c r="G310" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2025/2026</t>
+          <t>2025/2026, 2027/2028</t>
         </is>
       </c>
       <c r="H310" s="5" t="inlineStr">
@@ -15346,7 +15346,7 @@
       </c>
       <c r="G311" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2025/2026, 2026/2027</t>
+          <t>2025/2026, 2027/2028, 2026/2027</t>
         </is>
       </c>
       <c r="H311" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-07-19 23:52:16
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -9974,7 +9974,7 @@
       </c>
       <c r="G195" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 160715@med.asu.edu.eg</t>
+          <t>160715@med.asu.edu.eg, 2025/2026</t>
         </is>
       </c>
       <c r="H195" s="5" t="inlineStr">
@@ -11830,7 +11830,7 @@
       </c>
       <c r="G235" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 160715@med.asu.edu.eg</t>
+          <t>160715@med.asu.edu.eg, 2025/2026</t>
         </is>
       </c>
       <c r="H235" s="5" t="inlineStr">
@@ -13498,7 +13498,7 @@
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2027/2028, 2026/2027</t>
+          <t>2025/2026, 2026/2027, 2027/2028</t>
         </is>
       </c>
       <c r="H271" s="5" t="inlineStr">
@@ -15346,7 +15346,7 @@
       </c>
       <c r="G311" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2027/2028, 2026/2027</t>
+          <t>2025/2026, 2026/2027, 2027/2028</t>
         </is>
       </c>
       <c r="H311" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-07-21 17:10:27
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -9974,7 +9974,7 @@
       </c>
       <c r="G195" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 160715@med.asu.edu.eg</t>
+          <t>160715@med.asu.edu.eg, 2025/2026</t>
         </is>
       </c>
       <c r="H195" s="5" t="inlineStr">
@@ -11830,7 +11830,7 @@
       </c>
       <c r="G235" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 160715@med.asu.edu.eg</t>
+          <t>160715@med.asu.edu.eg, 2025/2026</t>
         </is>
       </c>
       <c r="H235" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-07-22 19:04:22
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -13451,7 +13451,7 @@
       </c>
       <c r="G270" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2025/2026</t>
+          <t>2025/2026, 2027/2028</t>
         </is>
       </c>
       <c r="H270" s="5" t="inlineStr">
@@ -13498,7 +13498,7 @@
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2025/2026, 2026/2027</t>
+          <t>2025/2026, 2026/2027, 2027/2028</t>
         </is>
       </c>
       <c r="H271" s="5" t="inlineStr">
@@ -15299,7 +15299,7 @@
       </c>
       <c r="G310" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2025/2026</t>
+          <t>2025/2026, 2027/2028</t>
         </is>
       </c>
       <c r="H310" s="5" t="inlineStr">
@@ -15346,7 +15346,7 @@
       </c>
       <c r="G311" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2025/2026, 2026/2027</t>
+          <t>2025/2026, 2026/2027, 2027/2028</t>
         </is>
       </c>
       <c r="H311" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-07-22 20:58:51
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -13498,7 +13498,7 @@
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2026/2027, 2027/2028</t>
+          <t>2025/2026, 2027/2028, 2026/2027</t>
         </is>
       </c>
       <c r="H271" s="5" t="inlineStr">
@@ -15346,7 +15346,7 @@
       </c>
       <c r="G311" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2026/2027, 2027/2028</t>
+          <t>2025/2026, 2027/2028, 2026/2027</t>
         </is>
       </c>
       <c r="H311" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-07-23 15:50:53
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -13498,7 +13498,7 @@
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>2026/2027, 2027/2028, 2025/2026</t>
+          <t>2027/2028, 2026/2027, 2025/2026</t>
         </is>
       </c>
       <c r="H271" s="5" t="inlineStr">
@@ -15346,7 +15346,7 @@
       </c>
       <c r="G311" s="5" t="inlineStr">
         <is>
-          <t>2026/2027, 2027/2028, 2025/2026</t>
+          <t>2027/2028, 2026/2027, 2025/2026</t>
         </is>
       </c>
       <c r="H311" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-07-24 05:44:13
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -9974,7 +9974,7 @@
       </c>
       <c r="G195" s="5" t="inlineStr">
         <is>
-          <t>160715@med.asu.edu.eg, 2025/2026</t>
+          <t>2025/2026, 160715@med.asu.edu.eg</t>
         </is>
       </c>
       <c r="H195" s="5" t="inlineStr">
@@ -11830,7 +11830,7 @@
       </c>
       <c r="G235" s="5" t="inlineStr">
         <is>
-          <t>160715@med.asu.edu.eg, 2025/2026</t>
+          <t>2025/2026, 160715@med.asu.edu.eg</t>
         </is>
       </c>
       <c r="H235" s="5" t="inlineStr">
@@ -13498,7 +13498,7 @@
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>2026/2027, 2025/2026, 2027/2028</t>
+          <t>2025/2026, 2026/2027, 2027/2028</t>
         </is>
       </c>
       <c r="H271" s="5" t="inlineStr">
@@ -15346,7 +15346,7 @@
       </c>
       <c r="G311" s="5" t="inlineStr">
         <is>
-          <t>2026/2027, 2025/2026, 2027/2028</t>
+          <t>2025/2026, 2026/2027, 2027/2028</t>
         </is>
       </c>
       <c r="H311" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-07-24 20:15:22
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -9974,7 +9974,7 @@
       </c>
       <c r="G195" s="5" t="inlineStr">
         <is>
-          <t>160715@med.asu.edu.eg, 2025/2026</t>
+          <t>2025/2026, 160715@med.asu.edu.eg</t>
         </is>
       </c>
       <c r="H195" s="5" t="inlineStr">
@@ -11830,7 +11830,7 @@
       </c>
       <c r="G235" s="5" t="inlineStr">
         <is>
-          <t>160715@med.asu.edu.eg, 2025/2026</t>
+          <t>2025/2026, 160715@med.asu.edu.eg</t>
         </is>
       </c>
       <c r="H235" s="5" t="inlineStr">
@@ -13451,7 +13451,7 @@
       </c>
       <c r="G270" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2025/2026</t>
+          <t>2025/2026, 2027/2028</t>
         </is>
       </c>
       <c r="H270" s="5" t="inlineStr">
@@ -13498,7 +13498,7 @@
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>2026/2027, 2027/2028, 2025/2026</t>
+          <t>2026/2027, 2025/2026, 2027/2028</t>
         </is>
       </c>
       <c r="H271" s="5" t="inlineStr">
@@ -15299,7 +15299,7 @@
       </c>
       <c r="G310" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2025/2026</t>
+          <t>2025/2026, 2027/2028</t>
         </is>
       </c>
       <c r="H310" s="5" t="inlineStr">
@@ -15346,7 +15346,7 @@
       </c>
       <c r="G311" s="5" t="inlineStr">
         <is>
-          <t>2026/2027, 2027/2028, 2025/2026</t>
+          <t>2026/2027, 2025/2026, 2027/2028</t>
         </is>
       </c>
       <c r="H311" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-07-27 22:00:20
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -13498,7 +13498,7 @@
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2026/2027, 2025/2026</t>
+          <t>2026/2027, 2027/2028, 2025/2026</t>
         </is>
       </c>
       <c r="H271" s="5" t="inlineStr">
@@ -15346,7 +15346,7 @@
       </c>
       <c r="G311" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2026/2027, 2025/2026</t>
+          <t>2026/2027, 2027/2028, 2025/2026</t>
         </is>
       </c>
       <c r="H311" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-07-28 23:58:16
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -13498,7 +13498,7 @@
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>2026/2027, 2027/2028, 2025/2026</t>
+          <t>2027/2028, 2026/2027, 2025/2026</t>
         </is>
       </c>
       <c r="H271" s="5" t="inlineStr">
@@ -15346,7 +15346,7 @@
       </c>
       <c r="G311" s="5" t="inlineStr">
         <is>
-          <t>2026/2027, 2027/2028, 2025/2026</t>
+          <t>2027/2028, 2026/2027, 2025/2026</t>
         </is>
       </c>
       <c r="H311" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-07-29 15:47:06
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -9974,7 +9974,7 @@
       </c>
       <c r="G195" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 160715@med.asu.edu.eg</t>
+          <t>160715@med.asu.edu.eg, 2025/2026</t>
         </is>
       </c>
       <c r="H195" s="5" t="inlineStr">
@@ -11830,7 +11830,7 @@
       </c>
       <c r="G235" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 160715@med.asu.edu.eg</t>
+          <t>160715@med.asu.edu.eg, 2025/2026</t>
         </is>
       </c>
       <c r="H235" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-07-30 19:16:09
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -9974,7 +9974,7 @@
       </c>
       <c r="G195" s="5" t="inlineStr">
         <is>
-          <t>160715@med.asu.edu.eg, 2025/2026</t>
+          <t>2025/2026, 160715@med.asu.edu.eg</t>
         </is>
       </c>
       <c r="H195" s="5" t="inlineStr">
@@ -11830,7 +11830,7 @@
       </c>
       <c r="G235" s="5" t="inlineStr">
         <is>
-          <t>160715@med.asu.edu.eg, 2025/2026</t>
+          <t>2025/2026, 160715@med.asu.edu.eg</t>
         </is>
       </c>
       <c r="H235" s="5" t="inlineStr">
@@ -13498,7 +13498,7 @@
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>2026/2027, 2027/2028, 2025/2026</t>
+          <t>2027/2028, 2026/2027, 2025/2026</t>
         </is>
       </c>
       <c r="H271" s="5" t="inlineStr">
@@ -15346,7 +15346,7 @@
       </c>
       <c r="G311" s="5" t="inlineStr">
         <is>
-          <t>2026/2027, 2027/2028, 2025/2026</t>
+          <t>2027/2028, 2026/2027, 2025/2026</t>
         </is>
       </c>
       <c r="H311" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-07-30 21:01:23
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -13451,7 +13451,7 @@
       </c>
       <c r="G270" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2025/2026</t>
+          <t>2025/2026, 2027/2028</t>
         </is>
       </c>
       <c r="H270" s="5" t="inlineStr">
@@ -13498,7 +13498,7 @@
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2026/2027, 2025/2026</t>
+          <t>2026/2027, 2025/2026, 2027/2028</t>
         </is>
       </c>
       <c r="H271" s="5" t="inlineStr">
@@ -15299,7 +15299,7 @@
       </c>
       <c r="G310" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2025/2026</t>
+          <t>2025/2026, 2027/2028</t>
         </is>
       </c>
       <c r="H310" s="5" t="inlineStr">
@@ -15346,7 +15346,7 @@
       </c>
       <c r="G311" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2026/2027, 2025/2026</t>
+          <t>2026/2027, 2025/2026, 2027/2028</t>
         </is>
       </c>
       <c r="H311" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-08-02 11:57:49
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -9974,7 +9974,7 @@
       </c>
       <c r="G195" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 160715@med.asu.edu.eg</t>
+          <t>160715@med.asu.edu.eg, 2025/2026</t>
         </is>
       </c>
       <c r="H195" s="5" t="inlineStr">
@@ -11830,7 +11830,7 @@
       </c>
       <c r="G235" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 160715@med.asu.edu.eg</t>
+          <t>160715@med.asu.edu.eg, 2025/2026</t>
         </is>
       </c>
       <c r="H235" s="5" t="inlineStr">
@@ -13451,7 +13451,7 @@
       </c>
       <c r="G270" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2027/2028</t>
+          <t>2027/2028, 2025/2026</t>
         </is>
       </c>
       <c r="H270" s="5" t="inlineStr">
@@ -13498,7 +13498,7 @@
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2026/2027, 2027/2028</t>
+          <t>2027/2028, 2025/2026, 2026/2027</t>
         </is>
       </c>
       <c r="H271" s="5" t="inlineStr">
@@ -15299,7 +15299,7 @@
       </c>
       <c r="G310" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2027/2028</t>
+          <t>2027/2028, 2025/2026</t>
         </is>
       </c>
       <c r="H310" s="5" t="inlineStr">
@@ -15346,7 +15346,7 @@
       </c>
       <c r="G311" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2026/2027, 2027/2028</t>
+          <t>2027/2028, 2025/2026, 2026/2027</t>
         </is>
       </c>
       <c r="H311" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-08-02 20:07:29
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -13451,7 +13451,7 @@
       </c>
       <c r="G270" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2025/2026</t>
+          <t>2025/2026, 2027/2028</t>
         </is>
       </c>
       <c r="H270" s="5" t="inlineStr">
@@ -13498,7 +13498,7 @@
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2025/2026, 2026/2027</t>
+          <t>2025/2026, 2027/2028, 2026/2027</t>
         </is>
       </c>
       <c r="H271" s="5" t="inlineStr">
@@ -15299,7 +15299,7 @@
       </c>
       <c r="G310" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2025/2026</t>
+          <t>2025/2026, 2027/2028</t>
         </is>
       </c>
       <c r="H310" s="5" t="inlineStr">
@@ -15346,7 +15346,7 @@
       </c>
       <c r="G311" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2025/2026, 2026/2027</t>
+          <t>2025/2026, 2027/2028, 2026/2027</t>
         </is>
       </c>
       <c r="H311" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-08-02 23:53:12
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -13451,7 +13451,7 @@
       </c>
       <c r="G270" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2027/2028</t>
+          <t>2027/2028, 2025/2026</t>
         </is>
       </c>
       <c r="H270" s="5" t="inlineStr">
@@ -13498,7 +13498,7 @@
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>2026/2027, 2025/2026, 2027/2028</t>
+          <t>2027/2028, 2026/2027, 2025/2026</t>
         </is>
       </c>
       <c r="H271" s="5" t="inlineStr">
@@ -15299,7 +15299,7 @@
       </c>
       <c r="G310" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2027/2028</t>
+          <t>2027/2028, 2025/2026</t>
         </is>
       </c>
       <c r="H310" s="5" t="inlineStr">
@@ -15346,7 +15346,7 @@
       </c>
       <c r="G311" s="5" t="inlineStr">
         <is>
-          <t>2026/2027, 2025/2026, 2027/2028</t>
+          <t>2027/2028, 2026/2027, 2025/2026</t>
         </is>
       </c>
       <c r="H311" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-08-03 18:45:50
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -13498,7 +13498,7 @@
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2025/2026, 2026/2027</t>
+          <t>2026/2027, 2027/2028, 2025/2026</t>
         </is>
       </c>
       <c r="H271" s="5" t="inlineStr">
@@ -15346,7 +15346,7 @@
       </c>
       <c r="G311" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2025/2026, 2026/2027</t>
+          <t>2026/2027, 2027/2028, 2025/2026</t>
         </is>
       </c>
       <c r="H311" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-08-05 02:55:00
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -9974,7 +9974,7 @@
       </c>
       <c r="G195" s="5" t="inlineStr">
         <is>
-          <t>160715@med.asu.edu.eg, 2025/2026</t>
+          <t>2025/2026, 160715@med.asu.edu.eg</t>
         </is>
       </c>
       <c r="H195" s="5" t="inlineStr">
@@ -11830,7 +11830,7 @@
       </c>
       <c r="G235" s="5" t="inlineStr">
         <is>
-          <t>160715@med.asu.edu.eg, 2025/2026</t>
+          <t>2025/2026, 160715@med.asu.edu.eg</t>
         </is>
       </c>
       <c r="H235" s="5" t="inlineStr">
@@ -13498,7 +13498,7 @@
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2027/2028, 2026/2027</t>
+          <t>2026/2027, 2025/2026, 2027/2028</t>
         </is>
       </c>
       <c r="H271" s="5" t="inlineStr">
@@ -15346,7 +15346,7 @@
       </c>
       <c r="G311" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2027/2028, 2026/2027</t>
+          <t>2026/2027, 2025/2026, 2027/2028</t>
         </is>
       </c>
       <c r="H311" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-08-05 13:52:58
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -9974,7 +9974,7 @@
       </c>
       <c r="G195" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 160715@med.asu.edu.eg</t>
+          <t>160715@med.asu.edu.eg, 2025/2026</t>
         </is>
       </c>
       <c r="H195" s="5" t="inlineStr">
@@ -11830,7 +11830,7 @@
       </c>
       <c r="G235" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 160715@med.asu.edu.eg</t>
+          <t>160715@med.asu.edu.eg, 2025/2026</t>
         </is>
       </c>
       <c r="H235" s="5" t="inlineStr">
@@ -13451,7 +13451,7 @@
       </c>
       <c r="G270" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2025/2026</t>
+          <t>2025/2026, 2027/2028</t>
         </is>
       </c>
       <c r="H270" s="5" t="inlineStr">
@@ -13498,7 +13498,7 @@
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2025/2026, 2026/2027</t>
+          <t>2025/2026, 2027/2028, 2026/2027</t>
         </is>
       </c>
       <c r="H271" s="5" t="inlineStr">
@@ -15299,7 +15299,7 @@
       </c>
       <c r="G310" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2025/2026</t>
+          <t>2025/2026, 2027/2028</t>
         </is>
       </c>
       <c r="H310" s="5" t="inlineStr">
@@ -15346,7 +15346,7 @@
       </c>
       <c r="G311" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2025/2026, 2026/2027</t>
+          <t>2025/2026, 2027/2028, 2026/2027</t>
         </is>
       </c>
       <c r="H311" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-08-05 15:58:20
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -9974,7 +9974,7 @@
       </c>
       <c r="G195" s="5" t="inlineStr">
         <is>
-          <t>160715@med.asu.edu.eg, 2025/2026</t>
+          <t>2025/2026, 160715@med.asu.edu.eg</t>
         </is>
       </c>
       <c r="H195" s="5" t="inlineStr">
@@ -11830,7 +11830,7 @@
       </c>
       <c r="G235" s="5" t="inlineStr">
         <is>
-          <t>160715@med.asu.edu.eg, 2025/2026</t>
+          <t>2025/2026, 160715@med.asu.edu.eg</t>
         </is>
       </c>
       <c r="H235" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-08-06 02:00:30
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -13498,7 +13498,7 @@
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2025/2026, 2026/2027</t>
+          <t>2027/2028, 2026/2027, 2025/2026</t>
         </is>
       </c>
       <c r="H271" s="5" t="inlineStr">
@@ -15346,7 +15346,7 @@
       </c>
       <c r="G311" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2025/2026, 2026/2027</t>
+          <t>2027/2028, 2026/2027, 2025/2026</t>
         </is>
       </c>
       <c r="H311" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-08-07 16:46:28
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -13498,7 +13498,7 @@
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>2026/2027, 2027/2028, 2025/2026</t>
+          <t>2027/2028, 2026/2027, 2025/2026</t>
         </is>
       </c>
       <c r="H271" s="5" t="inlineStr">
@@ -15346,7 +15346,7 @@
       </c>
       <c r="G311" s="5" t="inlineStr">
         <is>
-          <t>2026/2027, 2027/2028, 2025/2026</t>
+          <t>2027/2028, 2026/2027, 2025/2026</t>
         </is>
       </c>
       <c r="H311" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-08-08 12:34:58
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -9974,7 +9974,7 @@
       </c>
       <c r="G195" s="5" t="inlineStr">
         <is>
-          <t>160715@med.asu.edu.eg, 2025/2026</t>
+          <t>2025/2026, 160715@med.asu.edu.eg</t>
         </is>
       </c>
       <c r="H195" s="5" t="inlineStr">
@@ -11830,7 +11830,7 @@
       </c>
       <c r="G235" s="5" t="inlineStr">
         <is>
-          <t>160715@med.asu.edu.eg, 2025/2026</t>
+          <t>2025/2026, 160715@med.asu.edu.eg</t>
         </is>
       </c>
       <c r="H235" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-08-08 18:28:05
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -13498,7 +13498,7 @@
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2026/2027, 2027/2028</t>
+          <t>2026/2027, 2025/2026, 2027/2028</t>
         </is>
       </c>
       <c r="H271" s="5" t="inlineStr">
@@ -15346,7 +15346,7 @@
       </c>
       <c r="G311" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2026/2027, 2027/2028</t>
+          <t>2026/2027, 2025/2026, 2027/2028</t>
         </is>
       </c>
       <c r="H311" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-08-09 12:37:31
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -9974,7 +9974,7 @@
       </c>
       <c r="G195" s="5" t="inlineStr">
         <is>
-          <t>160715@med.asu.edu.eg, 2025/2026</t>
+          <t>2025/2026, 160715@med.asu.edu.eg</t>
         </is>
       </c>
       <c r="H195" s="5" t="inlineStr">
@@ -11830,7 +11830,7 @@
       </c>
       <c r="G235" s="5" t="inlineStr">
         <is>
-          <t>160715@med.asu.edu.eg, 2025/2026</t>
+          <t>2025/2026, 160715@med.asu.edu.eg</t>
         </is>
       </c>
       <c r="H235" s="5" t="inlineStr">
@@ -13498,7 +13498,7 @@
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2026/2027, 2027/2028</t>
+          <t>2026/2027, 2025/2026, 2027/2028</t>
         </is>
       </c>
       <c r="H271" s="5" t="inlineStr">
@@ -15346,7 +15346,7 @@
       </c>
       <c r="G311" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2026/2027, 2027/2028</t>
+          <t>2026/2027, 2025/2026, 2027/2028</t>
         </is>
       </c>
       <c r="H311" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-08-10 01:15:18
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -13451,7 +13451,7 @@
       </c>
       <c r="G270" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2025/2026</t>
+          <t>2025/2026, 2027/2028</t>
         </is>
       </c>
       <c r="H270" s="5" t="inlineStr">
@@ -13498,7 +13498,7 @@
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2026/2027, 2025/2026</t>
+          <t>2026/2027, 2025/2026, 2027/2028</t>
         </is>
       </c>
       <c r="H271" s="5" t="inlineStr">
@@ -15299,7 +15299,7 @@
       </c>
       <c r="G310" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2025/2026</t>
+          <t>2025/2026, 2027/2028</t>
         </is>
       </c>
       <c r="H310" s="5" t="inlineStr">
@@ -15346,7 +15346,7 @@
       </c>
       <c r="G311" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2026/2027, 2025/2026</t>
+          <t>2026/2027, 2025/2026, 2027/2028</t>
         </is>
       </c>
       <c r="H311" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-08-11 15:55:08
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -13498,7 +13498,7 @@
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2027/2028, 2026/2027</t>
+          <t>2025/2026, 2026/2027, 2027/2028</t>
         </is>
       </c>
       <c r="H271" s="5" t="inlineStr">
@@ -15346,7 +15346,7 @@
       </c>
       <c r="G311" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2027/2028, 2026/2027</t>
+          <t>2025/2026, 2026/2027, 2027/2028</t>
         </is>
       </c>
       <c r="H311" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-08-12 14:17:41
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -13498,7 +13498,7 @@
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2027/2028, 2026/2027</t>
+          <t>2025/2026, 2026/2027, 2027/2028</t>
         </is>
       </c>
       <c r="H271" s="5" t="inlineStr">
@@ -15346,7 +15346,7 @@
       </c>
       <c r="G311" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2027/2028, 2026/2027</t>
+          <t>2025/2026, 2026/2027, 2027/2028</t>
         </is>
       </c>
       <c r="H311" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-08-12 23:34:23
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -9974,7 +9974,7 @@
       </c>
       <c r="G195" s="5" t="inlineStr">
         <is>
-          <t>160715@med.asu.edu.eg, 2025/2026</t>
+          <t>2025/2026, 160715@med.asu.edu.eg</t>
         </is>
       </c>
       <c r="H195" s="5" t="inlineStr">
@@ -11830,7 +11830,7 @@
       </c>
       <c r="G235" s="5" t="inlineStr">
         <is>
-          <t>160715@med.asu.edu.eg, 2025/2026</t>
+          <t>2025/2026, 160715@med.asu.edu.eg</t>
         </is>
       </c>
       <c r="H235" s="5" t="inlineStr">

</xml_diff>